<commit_message>
Update historical price analysis 2026-09
</commit_message>
<xml_diff>
--- a/outputs/NSW_historical_prices.xlsx
+++ b/outputs/NSW_historical_prices.xlsx
@@ -528,16 +528,16 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>73.3</v>
+        <v>72.2</v>
       </c>
       <c r="C5" s="5" t="n">
-        <v>73.34999999999999</v>
+        <v>72.03</v>
       </c>
       <c r="D5" s="5" t="n">
-        <v>74.09</v>
+        <v>72.84</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>74.13</v>
+        <v>72.68000000000001</v>
       </c>
     </row>
     <row r="6">
@@ -550,13 +550,13 @@
         <v>96.44</v>
       </c>
       <c r="C6" s="5" t="n">
-        <v>114.4</v>
+        <v>114.45</v>
       </c>
       <c r="D6" s="5" t="n">
-        <v>99.66</v>
+        <v>99.52</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>118.46</v>
+        <v>118.4</v>
       </c>
     </row>
     <row r="7">
@@ -566,16 +566,16 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>101.61</v>
+        <v>101.43</v>
       </c>
       <c r="C7" s="5" t="n">
-        <v>123.47</v>
+        <v>122.92</v>
       </c>
       <c r="D7" s="5" t="n">
-        <v>106.36</v>
+        <v>106.02</v>
       </c>
       <c r="E7" s="5" t="n">
-        <v>129.43</v>
+        <v>128.71</v>
       </c>
     </row>
     <row r="8">
@@ -585,16 +585,16 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>116.19</v>
+        <v>116.34</v>
       </c>
       <c r="C8" s="5" t="n">
-        <v>134.55</v>
+        <v>134.6</v>
       </c>
       <c r="D8" s="5" t="n">
-        <v>127.5</v>
+        <v>127.46</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>147.39</v>
+        <v>147.25</v>
       </c>
     </row>
     <row r="9">
@@ -604,22 +604,22 @@
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>97.59999999999999</v>
+        <v>97.70999999999999</v>
       </c>
       <c r="C9" s="5" t="n">
         <v>114.84</v>
       </c>
       <c r="D9" s="5" t="n">
-        <v>114.84</v>
+        <v>114.82</v>
       </c>
       <c r="E9" s="5" t="n">
-        <v>135.15</v>
+        <v>135.01</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>Data through: Aug 2026</t>
+          <t>Data through: Sep 2026</t>
         </is>
       </c>
     </row>
@@ -634,7 +634,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F279"/>
+  <dimension ref="A1:F280"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6333,6 +6333,26 @@
       </c>
       <c r="F279" s="7" t="inlineStr"/>
     </row>
+    <row r="280">
+      <c r="A280" s="4" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="B280" s="5" t="n">
+        <v>58.08</v>
+      </c>
+      <c r="C280" s="5" t="n">
+        <v>50.65</v>
+      </c>
+      <c r="D280" s="5" t="n">
+        <v>58.08</v>
+      </c>
+      <c r="E280" s="5" t="n">
+        <v>50.65</v>
+      </c>
+      <c r="F280" s="7" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -6344,7 +6364,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E279"/>
+  <dimension ref="A1:E280"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -11663,8 +11683,27 @@
         <v>84.17</v>
       </c>
     </row>
+    <row r="280">
+      <c r="A280" s="4" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="B280" s="5" t="n">
+        <v>58.08</v>
+      </c>
+      <c r="C280" s="5" t="n">
+        <v>50.65</v>
+      </c>
+      <c r="D280" s="5" t="n">
+        <v>58.08</v>
+      </c>
+      <c r="E280" s="5" t="n">
+        <v>50.65</v>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="B2:B279">
+  <conditionalFormatting sqref="B2:B280">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -11676,7 +11715,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C2:C279">
+  <conditionalFormatting sqref="C2:C280">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
@@ -11688,7 +11727,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D2:D279">
+  <conditionalFormatting sqref="D2:D280">
     <cfRule type="colorScale" priority="3">
       <colorScale>
         <cfvo type="min"/>
@@ -11700,7 +11739,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E2:E279">
+  <conditionalFormatting sqref="E2:E280">
     <cfRule type="colorScale" priority="4">
       <colorScale>
         <cfvo type="min"/>

</xml_diff>

<commit_message>
Update historical price analysis 2026-10
</commit_message>
<xml_diff>
--- a/outputs/NSW_historical_prices.xlsx
+++ b/outputs/NSW_historical_prices.xlsx
@@ -528,16 +528,16 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>72.2</v>
+        <v>79.26000000000001</v>
       </c>
       <c r="C5" s="5" t="n">
-        <v>72.03</v>
+        <v>81.55</v>
       </c>
       <c r="D5" s="5" t="n">
-        <v>72.84</v>
+        <v>79.73999999999999</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>72.68000000000001</v>
+        <v>82.04000000000001</v>
       </c>
     </row>
     <row r="6">
@@ -547,16 +547,16 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>96.44</v>
+        <v>99.95</v>
       </c>
       <c r="C6" s="5" t="n">
-        <v>114.45</v>
+        <v>118.95</v>
       </c>
       <c r="D6" s="5" t="n">
-        <v>99.52</v>
+        <v>102.85</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>118.4</v>
+        <v>122.7</v>
       </c>
     </row>
     <row r="7">
@@ -566,16 +566,16 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>101.43</v>
+        <v>104.75</v>
       </c>
       <c r="C7" s="5" t="n">
-        <v>122.92</v>
+        <v>127.02</v>
       </c>
       <c r="D7" s="5" t="n">
-        <v>106.02</v>
+        <v>109.24</v>
       </c>
       <c r="E7" s="5" t="n">
-        <v>128.71</v>
+        <v>132.71</v>
       </c>
     </row>
     <row r="8">
@@ -585,16 +585,16 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>116.34</v>
+        <v>118.08</v>
       </c>
       <c r="C8" s="5" t="n">
-        <v>134.6</v>
+        <v>136.77</v>
       </c>
       <c r="D8" s="5" t="n">
-        <v>127.46</v>
+        <v>128.99</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>147.25</v>
+        <v>149.2</v>
       </c>
     </row>
     <row r="9">
@@ -604,22 +604,22 @@
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>97.70999999999999</v>
+        <v>98.59999999999999</v>
       </c>
       <c r="C9" s="5" t="n">
-        <v>114.84</v>
+        <v>115.91</v>
       </c>
       <c r="D9" s="5" t="n">
-        <v>114.82</v>
+        <v>115.55</v>
       </c>
       <c r="E9" s="5" t="n">
-        <v>135.01</v>
+        <v>135.91</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>Data through: Sep 2026</t>
+          <t>Data through: Oct 2026</t>
         </is>
       </c>
     </row>
@@ -634,7 +634,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F280"/>
+  <dimension ref="A1:F281"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6353,6 +6353,26 @@
       </c>
       <c r="F280" s="7" t="inlineStr"/>
     </row>
+    <row r="281">
+      <c r="A281" s="4" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="B281" s="5" t="n">
+        <v>161.68</v>
+      </c>
+      <c r="C281" s="5" t="n">
+        <v>189.53</v>
+      </c>
+      <c r="D281" s="5" t="n">
+        <v>161.68</v>
+      </c>
+      <c r="E281" s="5" t="n">
+        <v>189.53</v>
+      </c>
+      <c r="F281" s="7" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -6364,7 +6384,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E280"/>
+  <dimension ref="A1:E281"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -11702,8 +11722,27 @@
         <v>50.65</v>
       </c>
     </row>
+    <row r="281">
+      <c r="A281" s="4" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="B281" s="5" t="n">
+        <v>161.68</v>
+      </c>
+      <c r="C281" s="5" t="n">
+        <v>189.53</v>
+      </c>
+      <c r="D281" s="5" t="n">
+        <v>161.68</v>
+      </c>
+      <c r="E281" s="5" t="n">
+        <v>189.53</v>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="B2:B280">
+  <conditionalFormatting sqref="B2:B281">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -11715,7 +11754,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C2:C280">
+  <conditionalFormatting sqref="C2:C281">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
@@ -11727,7 +11766,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D2:D280">
+  <conditionalFormatting sqref="D2:D281">
     <cfRule type="colorScale" priority="3">
       <colorScale>
         <cfvo type="min"/>
@@ -11739,7 +11778,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E2:E280">
+  <conditionalFormatting sqref="E2:E281">
     <cfRule type="colorScale" priority="4">
       <colorScale>
         <cfvo type="min"/>

</xml_diff>